<commit_message>
Update smartcard (rename cancellationDate -> oppositionDate and rm date)  (#260)
* update smartcard

* update opposition date

* change oppositionDate short a865ed85f10bf10c468d34d8557509e0e1b79911
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-ext-smartcard.xlsx
+++ b/main/ig/StructureDefinition-as-ext-smartcard.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1180" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1017" uniqueCount="171">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-12T15:24:25+00:00</t>
+    <t>2025-03-18T14:02:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -518,43 +518,25 @@
     <t>./high</t>
   </si>
   <si>
-    <t>Extension.extension:cancellationDate</t>
-  </si>
-  <si>
-    <t>cancellationDate</t>
-  </si>
-  <si>
-    <t>dateOpposition : Date de mise en opposition de la carte.</t>
-  </si>
-  <si>
-    <t>Extension.extension:cancellationDate.id</t>
-  </si>
-  <si>
-    <t>Extension.extension:cancellationDate.extension</t>
-  </si>
-  <si>
-    <t>Extension.extension:cancellationDate.url</t>
-  </si>
-  <si>
-    <t>Extension.extension:cancellationDate.value[x]</t>
-  </si>
-  <si>
-    <t>Extension.extension:date</t>
-  </si>
-  <si>
-    <t>date</t>
-  </si>
-  <si>
-    <t>Extension.extension:date.id</t>
-  </si>
-  <si>
-    <t>Extension.extension:date.extension</t>
-  </si>
-  <si>
-    <t>Extension.extension:date.url</t>
-  </si>
-  <si>
-    <t>Extension.extension:date.value[x]</t>
+    <t>Extension.extension:oppositionDate</t>
+  </si>
+  <si>
+    <t>oppositionDate</t>
+  </si>
+  <si>
+    <t>dateOpposition : Date d'opposition de la carte.</t>
+  </si>
+  <si>
+    <t>Extension.extension:oppositionDate.id</t>
+  </si>
+  <si>
+    <t>Extension.extension:oppositionDate.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension:oppositionDate.url</t>
+  </si>
+  <si>
+    <t>Extension.extension:oppositionDate.value[x]</t>
   </si>
   <si>
     <t>base64Binary
@@ -868,12 +850,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK35"/>
+  <dimension ref="A1:AK30"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="45.23046875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="43.71484375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="37.25390625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="16.5078125" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="14.97265625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="12.64453125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="6.77734375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.9453125" customWidth="true" bestFit="true"/>
@@ -3829,23 +3811,21 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>170</v>
+        <v>114</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="C29" t="s" s="2">
-        <v>171</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="G29" t="s" s="2">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="H29" t="s" s="2">
         <v>76</v>
@@ -3857,22 +3837,24 @@
         <v>76</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>30</v>
+        <v>111</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>103</v>
-      </c>
-      <c r="N29" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="N29" t="s" s="2">
+        <v>113</v>
+      </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q29" s="2"/>
       <c r="R29" t="s" s="2">
-        <v>76</v>
+        <v>3</v>
       </c>
       <c r="S29" t="s" s="2">
         <v>76</v>
@@ -3914,30 +3896,30 @@
         <v>76</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="AG29" t="s" s="2">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>76</v>
+        <v>115</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>172</v>
+        <v>123</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>105</v>
+        <v>123</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -3948,7 +3930,7 @@
         <v>77</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="H30" t="s" s="2">
         <v>76</v>
@@ -3960,13 +3942,13 @@
         <v>76</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>85</v>
+        <v>170</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>87</v>
+        <v>120</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -4017,7 +3999,7 @@
         <v>76</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>88</v>
+        <v>123</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>77</v>
@@ -4029,530 +4011,9 @@
         <v>76</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>76</v>
+        <v>124</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="s" s="2">
-        <v>173</v>
-      </c>
-      <c r="B31" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="C31" s="2"/>
-      <c r="D31" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="E31" s="2"/>
-      <c r="F31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G31" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="H31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="I31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="J31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="K31" t="s" s="2">
-        <v>92</v>
-      </c>
-      <c r="L31" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="M31" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="N31" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="O31" s="2"/>
-      <c r="P31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Q31" s="2"/>
-      <c r="R31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="S31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="T31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="U31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="V31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="W31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="X31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Z31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AA31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AB31" t="s" s="2">
-        <v>96</v>
-      </c>
-      <c r="AC31" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="AD31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AE31" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="AF31" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AG31" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH31" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AI31" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ31" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AK31" t="s" s="2">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="B32" t="s" s="2">
-        <v>109</v>
-      </c>
-      <c r="C32" s="2"/>
-      <c r="D32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="E32" s="2"/>
-      <c r="F32" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="G32" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="I32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="J32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="K32" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="L32" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="M32" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="N32" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="O32" s="2"/>
-      <c r="P32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Q32" s="2"/>
-      <c r="R32" t="s" s="2">
-        <v>171</v>
-      </c>
-      <c r="S32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="T32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="U32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="V32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="W32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="X32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Z32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AA32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AB32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AC32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AD32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AE32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AF32" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="AG32" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH32" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ32" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK32" t="s" s="2">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="s" s="2">
-        <v>175</v>
-      </c>
-      <c r="B33" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="C33" s="2"/>
-      <c r="D33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="E33" s="2"/>
-      <c r="F33" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G33" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="I33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="J33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="K33" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="L33" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="M33" t="s" s="2">
-        <v>120</v>
-      </c>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
-      <c r="P33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Q33" s="2"/>
-      <c r="R33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="S33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="T33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="U33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="V33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="W33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="X33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Z33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AA33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AB33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AC33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AD33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AE33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AF33" t="s" s="2">
-        <v>123</v>
-      </c>
-      <c r="AG33" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH33" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI33" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ33" t="s" s="2">
-        <v>124</v>
-      </c>
-      <c r="AK33" t="s" s="2">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="B34" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="C34" s="2"/>
-      <c r="D34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="E34" s="2"/>
-      <c r="F34" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="G34" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="H34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="I34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="J34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="K34" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="L34" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="M34" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="O34" s="2"/>
-      <c r="P34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Q34" s="2"/>
-      <c r="R34" t="s" s="2">
-        <v>3</v>
-      </c>
-      <c r="S34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="T34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="U34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="V34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="W34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="X34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Z34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AA34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AB34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AC34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AD34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AE34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AF34" t="s" s="2">
-        <v>114</v>
-      </c>
-      <c r="AG34" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AH34" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ34" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AK34" t="s" s="2">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="s" s="2">
-        <v>123</v>
-      </c>
-      <c r="B35" t="s" s="2">
-        <v>123</v>
-      </c>
-      <c r="C35" s="2"/>
-      <c r="D35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="E35" s="2"/>
-      <c r="F35" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="G35" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="H35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="I35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="J35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="K35" t="s" s="2">
-        <v>176</v>
-      </c>
-      <c r="L35" t="s" s="2">
-        <v>119</v>
-      </c>
-      <c r="M35" t="s" s="2">
-        <v>120</v>
-      </c>
-      <c r="N35" s="2"/>
-      <c r="O35" s="2"/>
-      <c r="P35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Q35" s="2"/>
-      <c r="R35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="S35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="T35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="U35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="V35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="W35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="X35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Y35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="Z35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AA35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AB35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AC35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AD35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AE35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AF35" t="s" s="2">
-        <v>123</v>
-      </c>
-      <c r="AG35" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH35" t="s" s="2">
-        <v>84</v>
-      </c>
-      <c r="AI35" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ35" t="s" s="2">
-        <v>124</v>
-      </c>
-      <c r="AK35" t="s" s="2">
         <v>115</v>
       </c>
     </row>

</xml_diff>